<commit_message>
Fixes the negative validation results.
</commit_message>
<xml_diff>
--- a/rules/CORE-000717/negative/01/data/unit-test-coreid-FB3401-negative.xlsx
+++ b/rules/CORE-000717/negative/01/data/unit-test-coreid-FB3401-negative.xlsx
@@ -54,16 +54,16 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
       <color rgb="FF000000"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
       <i/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <sz val="11"/>
@@ -131,8 +131,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -478,18 +478,18 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="4" t="str">
         <v>sdtmig</v>
       </c>
-      <c r="B2" s="4" t="str">
+      <c r="B2" s="5" t="str">
         <v>3-4</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="str">
+      <c r="A3" s="4" t="str">
         <v/>
       </c>
-      <c r="B3" s="4" t="str">
+      <c r="B3" s="5" t="str">
         <v/>
       </c>
     </row>
@@ -513,18 +513,18 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="str">
+      <c r="A2" s="4" t="str">
         <v>ae.xpt</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="4" t="str">
         <v>Adverse Events</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="str">
+      <c r="A3" s="4" t="str">
         <v>ds.xpt</v>
       </c>
-      <c r="B3" s="2" t="str">
+      <c r="B3" s="4" t="str">
         <v>Disposition</v>
       </c>
     </row>
@@ -560,42 +560,42 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2">
+      <c r="A2" s="4">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="str">
+      <c r="B2" s="4" t="str">
         <v>ae.xpt</v>
       </c>
-      <c r="C2" s="2" t="str">
+      <c r="C2" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="4">
         <v>7</v>
       </c>
-      <c r="E2" s="2" t="str">
+      <c r="E2" s="4" t="str">
         <v>AESTDTC</v>
       </c>
-      <c r="F2" s="2" t="str">
+      <c r="F2" s="4" t="str">
         <v>2022-02-20</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2">
+      <c r="A3" s="4">
         <v>1</v>
       </c>
-      <c r="B3" s="2" t="str">
+      <c r="B3" s="4" t="str">
         <v>ae.xpt</v>
       </c>
-      <c r="C3" s="2" t="str">
+      <c r="C3" s="4" t="str">
         <v>Record</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="4">
         <v>7</v>
       </c>
-      <c r="E3" s="2" t="str">
+      <c r="E3" s="4" t="str">
         <v>$max_dsstdtc</v>
       </c>
-      <c r="F3" s="2" t="str">
+      <c r="F3" s="4" t="str">
         <v>2022-01-19</v>
       </c>
     </row>
@@ -643,185 +643,185 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="str">
+      <c r="A2" s="6" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="5" t="str">
+      <c r="B2" s="6" t="str">
         <v>Domain Abbreviation</v>
       </c>
-      <c r="C2" s="5" t="str">
+      <c r="C2" s="6" t="str">
         <v>Unique Subject Identifier</v>
       </c>
-      <c r="D2" s="5" t="str">
+      <c r="D2" s="6" t="str">
         <v>Sequence Number</v>
       </c>
-      <c r="E2" s="5" t="str">
+      <c r="E2" s="6" t="str">
         <v>Reported Term for the Adverse Event</v>
       </c>
-      <c r="F2" s="5" t="str">
+      <c r="F2" s="6" t="str">
         <v>Serious Event</v>
       </c>
-      <c r="G2" s="5" t="str">
+      <c r="G2" s="6" t="str">
         <v>Outcome of Adverse Event</v>
       </c>
-      <c r="H2" s="5" t="str">
+      <c r="H2" s="6" t="str">
         <v xml:space="preserve">Results in Death </v>
       </c>
-      <c r="I2" s="5" t="str">
+      <c r="I2" s="6" t="str">
         <v>Start Date/Time of Adverse Event</v>
       </c>
-      <c r="J2" s="5" t="str">
+      <c r="J2" s="6" t="str">
         <v>End Date/Time of Adverse Event</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="B3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="C3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="D3" s="5" t="str">
+      <c r="A3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="B3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="C3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="D3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="E3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="F3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="G3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="H3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="I3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="J3" s="5" t="str">
+      <c r="E3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="F3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="G3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="H3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="I3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="J3" s="6" t="str">
         <v>Char</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5">
+      <c r="A4" s="6">
         <v>12</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B4" s="6">
         <v>2</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="6">
         <v>8</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="6">
         <v>8</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="6">
         <v>40</v>
       </c>
-      <c r="F4" s="5" t="str">
+      <c r="F4" s="6" t="str">
         <v>1</v>
       </c>
-      <c r="G4" s="5" t="str">
+      <c r="G4" s="6" t="str">
         <v>40</v>
       </c>
-      <c r="H4" s="5" t="str">
+      <c r="H4" s="6" t="str">
         <v>1</v>
       </c>
-      <c r="I4" s="5" t="str">
+      <c r="I4" s="6" t="str">
         <v>19</v>
       </c>
-      <c r="J4" s="5" t="str">
+      <c r="J4" s="6" t="str">
         <v>19</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B5" s="4" t="str">
+      <c r="A5" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B5" s="5" t="str">
         <v>AE</v>
       </c>
-      <c r="C5" s="6" t="str">
+      <c r="C5" s="4" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D5" s="6" t="str">
+      <c r="D5" s="4" t="str">
         <v>1</v>
       </c>
-      <c r="E5" s="4" t="str">
+      <c r="E5" s="5" t="str">
         <v>INFUSION ASSOCIATE REACTION</v>
       </c>
-      <c r="F5" s="4" t="str">
+      <c r="F5" s="5" t="str">
         <v>N</v>
       </c>
-      <c r="G5" s="4" t="str">
+      <c r="G5" s="5" t="str">
         <v>NOT RECOVERED/NOT RESOLVED</v>
       </c>
-      <c r="H5" s="4" t="str">
+      <c r="H5" s="5" t="str">
         <v/>
       </c>
-      <c r="I5" s="4" t="str">
+      <c r="I5" s="5" t="str">
         <v>2018-02-20</v>
       </c>
-      <c r="J5" s="4" t="str">
+      <c r="J5" s="5" t="str">
         <v>2018-02-20</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B6" s="4" t="str">
+      <c r="A6" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B6" s="5" t="str">
         <v>AE</v>
       </c>
-      <c r="C6" s="6" t="str">
+      <c r="C6" s="4" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D6" s="6" t="str">
+      <c r="D6" s="4" t="str">
         <v>2</v>
       </c>
-      <c r="E6" s="4" t="str">
+      <c r="E6" s="5" t="str">
         <v>INSOMNIA</v>
       </c>
-      <c r="F6" s="4" t="str">
+      <c r="F6" s="5" t="str">
         <v>N</v>
       </c>
-      <c r="G6" s="4" t="str">
+      <c r="G6" s="5" t="str">
         <v>RECOVERED/RESOLVED</v>
       </c>
-      <c r="H6" s="4" t="str">
+      <c r="H6" s="5" t="str">
         <v/>
       </c>
-      <c r="I6" s="4" t="str">
+      <c r="I6" s="5" t="str">
         <v>2018-02-22</v>
       </c>
-      <c r="J6" s="4" t="str">
+      <c r="J6" s="5" t="str">
         <v>2018-10-30</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B7" s="4" t="str">
+      <c r="A7" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B7" s="5" t="str">
         <v>AE</v>
       </c>
-      <c r="C7" s="6" t="str">
+      <c r="C7" s="4" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D7" s="6" t="str">
+      <c r="D7" s="4" t="str">
         <v>3</v>
       </c>
-      <c r="E7" s="4" t="str">
+      <c r="E7" s="5" t="str">
         <v>LETHARGY</v>
       </c>
-      <c r="F7" s="4" t="str">
+      <c r="F7" s="5" t="str">
         <v>N</v>
       </c>
-      <c r="G7" s="4" t="str">
+      <c r="G7" s="5" t="str">
         <v>RECOVERED/RESOLVED</v>
       </c>
       <c r="H7" s="7" t="str">
@@ -830,103 +830,103 @@
       <c r="I7" s="8" t="str">
         <v>2022-02-20</v>
       </c>
-      <c r="J7" s="4" t="str">
+      <c r="J7" s="5" t="str">
         <v>2018-06-12</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B8" s="4" t="str">
+      <c r="A8" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B8" s="5" t="str">
         <v>AE</v>
       </c>
-      <c r="C8" s="6" t="str">
+      <c r="C8" s="4" t="str">
         <v>CDISC002</v>
       </c>
-      <c r="D8" s="6" t="str">
+      <c r="D8" s="4" t="str">
         <v>1</v>
       </c>
-      <c r="E8" s="4" t="str">
+      <c r="E8" s="5" t="str">
         <v>FATIGUE</v>
       </c>
-      <c r="F8" s="4" t="str">
+      <c r="F8" s="5" t="str">
         <v>N</v>
       </c>
-      <c r="G8" s="4" t="str">
+      <c r="G8" s="5" t="str">
         <v>RECOVERED/RESOLVED</v>
       </c>
-      <c r="H8" s="4" t="str">
+      <c r="H8" s="5" t="str">
         <v/>
       </c>
-      <c r="I8" s="4" t="str">
+      <c r="I8" s="5" t="str">
         <v>2018-05-02</v>
       </c>
-      <c r="J8" s="4" t="str">
+      <c r="J8" s="5" t="str">
         <v>2018-10-22</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B9" s="4" t="str">
+      <c r="A9" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B9" s="5" t="str">
         <v>AE</v>
       </c>
-      <c r="C9" s="6" t="str">
+      <c r="C9" s="4" t="str">
         <v>CDISC002</v>
       </c>
-      <c r="D9" s="6" t="str">
+      <c r="D9" s="4" t="str">
         <v>2</v>
       </c>
-      <c r="E9" s="4" t="str">
+      <c r="E9" s="5" t="str">
         <v>CRAMPS (UNKNOWN LOCATION)</v>
       </c>
-      <c r="F9" s="4" t="str">
+      <c r="F9" s="5" t="str">
         <v>N</v>
       </c>
-      <c r="G9" s="4" t="str">
+      <c r="G9" s="5" t="str">
         <v>RECOVERED/RESOLVED</v>
       </c>
-      <c r="H9" s="4" t="str">
+      <c r="H9" s="5" t="str">
         <v/>
       </c>
-      <c r="I9" s="4" t="str">
+      <c r="I9" s="5" t="str">
         <v>2018-04</v>
       </c>
-      <c r="J9" s="4" t="str">
+      <c r="J9" s="5" t="str">
         <v>2019-03</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B10" s="4" t="str">
+      <c r="A10" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B10" s="5" t="str">
         <v>AE</v>
       </c>
-      <c r="C10" s="6" t="str">
+      <c r="C10" s="4" t="str">
         <v>CDISC002</v>
       </c>
-      <c r="D10" s="6" t="str">
+      <c r="D10" s="4" t="str">
         <v>3</v>
       </c>
-      <c r="E10" s="4" t="str">
+      <c r="E10" s="5" t="str">
         <v>LEFT HIP PAIN</v>
       </c>
-      <c r="F10" s="4" t="str">
+      <c r="F10" s="5" t="str">
         <v>N</v>
       </c>
-      <c r="G10" s="4" t="str">
+      <c r="G10" s="5" t="str">
         <v>RECOVERED/RESOLVED</v>
       </c>
       <c r="H10" s="9" t="str">
         <v/>
       </c>
-      <c r="I10" s="4" t="str">
+      <c r="I10" s="5" t="str">
         <v>2019-01-14</v>
       </c>
-      <c r="J10" s="4" t="str">
+      <c r="J10" s="5" t="str">
         <v>2018-09-04</v>
       </c>
     </row>
@@ -971,379 +971,379 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="str">
+      <c r="A2" s="6" t="str">
         <v>Study Identifier</v>
       </c>
-      <c r="B2" s="5" t="str">
+      <c r="B2" s="6" t="str">
         <v>Domain Abbreviation</v>
       </c>
-      <c r="C2" s="5" t="str">
+      <c r="C2" s="6" t="str">
         <v>Unique Subject Identifier</v>
       </c>
-      <c r="D2" s="5" t="str">
+      <c r="D2" s="6" t="str">
         <v>Sequence Number</v>
       </c>
-      <c r="E2" s="5" t="str">
+      <c r="E2" s="6" t="str">
         <v>Reported Term for the Adverse Event</v>
       </c>
-      <c r="F2" s="5" t="str">
+      <c r="F2" s="6" t="str">
         <v>Standardized Disposition Term</v>
       </c>
-      <c r="G2" s="5" t="str">
+      <c r="G2" s="6" t="str">
         <v>Category for Disposition Event</v>
       </c>
-      <c r="H2" s="5" t="str">
+      <c r="H2" s="6" t="str">
         <v>Epoch</v>
       </c>
-      <c r="I2" s="5" t="str">
+      <c r="I2" s="6" t="str">
         <v>Start Date/Time of Disposition Event</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="B3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="C3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="D3" s="5" t="str">
+      <c r="A3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="B3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="C3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="D3" s="6" t="str">
         <v>Num</v>
       </c>
-      <c r="E3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="F3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="G3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="H3" s="5" t="str">
-        <v>Char</v>
-      </c>
-      <c r="I3" s="5" t="str">
+      <c r="E3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="F3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="G3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="H3" s="6" t="str">
+        <v>Char</v>
+      </c>
+      <c r="I3" s="6" t="str">
         <v>Char</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5">
+      <c r="A4" s="6">
         <v>12</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B4" s="6">
         <v>2</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="6">
         <v>8</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="6">
         <v>8</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="6">
         <v>200</v>
       </c>
-      <c r="F4" s="5" t="str">
+      <c r="F4" s="6" t="str">
         <v>40</v>
       </c>
-      <c r="G4" s="5" t="str">
+      <c r="G4" s="6" t="str">
         <v>50</v>
       </c>
-      <c r="H4" s="5" t="str">
+      <c r="H4" s="6" t="str">
         <v>50</v>
       </c>
-      <c r="I4" s="5" t="str">
+      <c r="I4" s="6" t="str">
         <v>19</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B5" s="4" t="str">
+      <c r="A5" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B5" s="5" t="str">
         <v>DS</v>
       </c>
-      <c r="C5" s="6" t="str">
+      <c r="C5" s="4" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D5" s="6" t="str">
+      <c r="D5" s="4" t="str">
         <v>1</v>
       </c>
-      <c r="E5" s="2" t="str">
+      <c r="E5" s="4" t="str">
         <v>INFORMED CONSENT OBTAINED</v>
       </c>
-      <c r="F5" s="2" t="str">
+      <c r="F5" s="4" t="str">
         <v>INFORMED CONSENT OBTAINED</v>
       </c>
-      <c r="G5" s="2" t="str">
+      <c r="G5" s="4" t="str">
         <v>PROTOCOL MILESTONE</v>
       </c>
-      <c r="H5" s="2" t="str">
+      <c r="H5" s="4" t="str">
         <v>SCREENING</v>
       </c>
-      <c r="I5" s="4" t="str">
+      <c r="I5" s="5" t="str">
         <v>2018-01-24</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B6" s="4" t="str">
+      <c r="A6" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B6" s="5" t="str">
         <v>DS</v>
       </c>
-      <c r="C6" s="6" t="str">
+      <c r="C6" s="4" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D6" s="6" t="str">
+      <c r="D6" s="4" t="str">
         <v>2</v>
       </c>
-      <c r="E6" s="2" t="str">
+      <c r="E6" s="4" t="str">
         <v>COMPLETED</v>
       </c>
-      <c r="F6" s="2" t="str">
+      <c r="F6" s="4" t="str">
         <v>COMPLETED</v>
       </c>
-      <c r="G6" s="2" t="str">
+      <c r="G6" s="4" t="str">
         <v>DISPOSITION EVENT</v>
       </c>
-      <c r="H6" s="2" t="str">
+      <c r="H6" s="4" t="str">
         <v>SCREENING</v>
       </c>
-      <c r="I6" s="4" t="str">
+      <c r="I6" s="5" t="str">
         <v>2018-02-15</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B7" s="4" t="str">
+      <c r="A7" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B7" s="5" t="str">
         <v>DS</v>
       </c>
-      <c r="C7" s="6" t="str">
+      <c r="C7" s="4" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D7" s="6" t="str">
+      <c r="D7" s="4" t="str">
         <v>3</v>
       </c>
-      <c r="E7" s="2" t="str">
+      <c r="E7" s="4" t="str">
         <v>RANDOMIZED</v>
       </c>
-      <c r="F7" s="2" t="str">
+      <c r="F7" s="4" t="str">
         <v>RANDOMIZED</v>
       </c>
-      <c r="G7" s="2" t="str">
+      <c r="G7" s="4" t="str">
         <v>PROTOCOL MILESTONE</v>
       </c>
-      <c r="H7" s="2" t="str">
+      <c r="H7" s="4" t="str">
         <v>SCREENING</v>
       </c>
-      <c r="I7" s="4" t="str">
+      <c r="I7" s="5" t="str">
         <v>2018-02-15T17:38</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B8" s="4" t="str">
+      <c r="A8" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B8" s="5" t="str">
         <v>DS</v>
       </c>
-      <c r="C8" s="6" t="str">
+      <c r="C8" s="4" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D8" s="6" t="str">
+      <c r="D8" s="4" t="str">
         <v>4</v>
       </c>
-      <c r="E8" s="2" t="str">
+      <c r="E8" s="4" t="str">
         <v>PROGRESSIVE DISEASE</v>
       </c>
-      <c r="F8" s="2" t="str">
+      <c r="F8" s="4" t="str">
         <v>PROGRESSIVE DISEASE</v>
       </c>
-      <c r="G8" s="2" t="str">
+      <c r="G8" s="4" t="str">
         <v>DISPOSITION EVENT</v>
       </c>
-      <c r="H8" s="2" t="str">
+      <c r="H8" s="4" t="str">
         <v>TREATMENT</v>
       </c>
-      <c r="I8" s="4" t="str">
+      <c r="I8" s="5" t="str">
         <v>2019-02-20</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B9" s="4" t="str">
+      <c r="A9" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B9" s="5" t="str">
         <v>DS</v>
       </c>
-      <c r="C9" s="6" t="str">
+      <c r="C9" s="4" t="str">
         <v>CDISC001</v>
       </c>
-      <c r="D9" s="6" t="str">
+      <c r="D9" s="4" t="str">
         <v>5</v>
       </c>
-      <c r="E9" s="2" t="str">
+      <c r="E9" s="4" t="str">
         <v>ALIVE</v>
       </c>
-      <c r="F9" s="4" t="str">
+      <c r="F9" s="5" t="str">
         <v>LAST CONTACT</v>
       </c>
-      <c r="G9" s="2" t="str">
+      <c r="G9" s="4" t="str">
         <v>DISPOSITION EVENT</v>
       </c>
-      <c r="H9" s="2" t="str">
+      <c r="H9" s="4" t="str">
         <v>FOLLOW-UP</v>
       </c>
-      <c r="I9" s="8" t="str">
+      <c r="I9" s="5" t="str">
         <v>2022-01-19</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B10" s="4" t="str">
+      <c r="A10" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B10" s="5" t="str">
         <v>DS</v>
       </c>
-      <c r="C10" s="6" t="str">
+      <c r="C10" s="4" t="str">
         <v>CDISC002</v>
       </c>
-      <c r="D10" s="6" t="str">
+      <c r="D10" s="4" t="str">
         <v>1</v>
       </c>
-      <c r="E10" s="2" t="str">
+      <c r="E10" s="4" t="str">
         <v>INFORMED CONSENT OBTAINED</v>
       </c>
-      <c r="F10" s="2" t="str">
+      <c r="F10" s="4" t="str">
         <v>INFORMED CONSENT OBTAINED</v>
       </c>
-      <c r="G10" s="2" t="str">
+      <c r="G10" s="4" t="str">
         <v>PROTOCOL MILESTONE</v>
       </c>
-      <c r="H10" s="2" t="str">
+      <c r="H10" s="4" t="str">
         <v>SCREENING</v>
       </c>
-      <c r="I10" s="4" t="str">
+      <c r="I10" s="5" t="str">
         <v>2018-03-22</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B11" s="4" t="str">
+      <c r="A11" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B11" s="5" t="str">
         <v>DS</v>
       </c>
-      <c r="C11" s="6" t="str">
+      <c r="C11" s="4" t="str">
         <v>CDISC002</v>
       </c>
-      <c r="D11" s="6" t="str">
+      <c r="D11" s="4" t="str">
         <v>2</v>
       </c>
-      <c r="E11" s="2" t="str">
+      <c r="E11" s="4" t="str">
         <v>COMPLETED</v>
       </c>
-      <c r="F11" s="2" t="str">
+      <c r="F11" s="4" t="str">
         <v>COMPLETED</v>
       </c>
-      <c r="G11" s="2" t="str">
+      <c r="G11" s="4" t="str">
         <v>DISPOSITION EVENT</v>
       </c>
-      <c r="H11" s="2" t="str">
+      <c r="H11" s="4" t="str">
         <v>SCREENING</v>
       </c>
-      <c r="I11" s="4" t="str">
+      <c r="I11" s="5" t="str">
         <v>2018-04-13</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="6" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B12" s="4" t="str">
+      <c r="A12" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B12" s="5" t="str">
         <v>DS</v>
       </c>
-      <c r="C12" s="6" t="str">
+      <c r="C12" s="4" t="str">
         <v>CDISC002</v>
       </c>
-      <c r="D12" s="6" t="str">
+      <c r="D12" s="4" t="str">
         <v>3</v>
       </c>
-      <c r="E12" s="2" t="str">
+      <c r="E12" s="4" t="str">
         <v>RANDOMIZED</v>
       </c>
-      <c r="F12" s="2" t="str">
+      <c r="F12" s="4" t="str">
         <v>RANDOMIZED</v>
       </c>
-      <c r="G12" s="2" t="str">
+      <c r="G12" s="4" t="str">
         <v>PROTOCOL MILESTONE</v>
       </c>
-      <c r="H12" s="2" t="str">
+      <c r="H12" s="4" t="str">
         <v>SCREENING</v>
       </c>
-      <c r="I12" s="4" t="str">
+      <c r="I12" s="5" t="str">
         <v>2018-04-13T13:09</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B13" s="4" t="str">
+      <c r="A13" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B13" s="5" t="str">
         <v>DS</v>
       </c>
-      <c r="C13" s="6" t="str">
+      <c r="C13" s="4" t="str">
         <v>CDISC002</v>
       </c>
-      <c r="D13" s="6" t="str">
+      <c r="D13" s="4" t="str">
         <v>4</v>
       </c>
-      <c r="E13" s="2" t="str">
+      <c r="E13" s="4" t="str">
         <v>ADVERSE EVENT</v>
       </c>
-      <c r="F13" s="2" t="str">
+      <c r="F13" s="4" t="str">
         <v>ADVERSE EVENT</v>
       </c>
-      <c r="G13" s="2" t="str">
+      <c r="G13" s="4" t="str">
         <v>DISPOSITION EVENT</v>
       </c>
-      <c r="H13" s="2" t="str">
+      <c r="H13" s="4" t="str">
         <v>TREATMENT</v>
       </c>
-      <c r="I13" s="4" t="str">
+      <c r="I13" s="5" t="str">
         <v>2019-01-30</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="str">
-        <v>CDISCPILOT01</v>
-      </c>
-      <c r="B14" s="4" t="str">
+      <c r="A14" s="4" t="str">
+        <v>CDISCPILOT01</v>
+      </c>
+      <c r="B14" s="5" t="str">
         <v>DS</v>
       </c>
-      <c r="C14" s="6" t="str">
+      <c r="C14" s="4" t="str">
         <v>CDISC002</v>
       </c>
-      <c r="D14" s="6" t="str">
+      <c r="D14" s="4" t="str">
         <v>5</v>
       </c>
-      <c r="E14" s="2" t="str">
+      <c r="E14" s="4" t="str">
         <v>PROGRESSIVE DISEASE</v>
       </c>
-      <c r="F14" s="2" t="str">
+      <c r="F14" s="4" t="str">
         <v>PROGRESSIVE DISEASE</v>
       </c>
-      <c r="G14" s="2" t="str">
+      <c r="G14" s="4" t="str">
         <v>DISPOSITION EVENT</v>
       </c>
-      <c r="H14" s="2" t="str">
+      <c r="H14" s="4" t="str">
         <v>FOLLOW-UP</v>
       </c>
-      <c r="I14" s="4" t="str">
+      <c r="I14" s="5" t="str">
         <v>2019-03-13</v>
       </c>
     </row>

</xml_diff>